<commit_message>
clean workflow - sna and tax
</commit_message>
<xml_diff>
--- a/input_data/admin_data/COL/_clean/total-pos-COL.xlsx
+++ b/input_data/admin_data/COL/_clean/total-pos-COL.xlsx
@@ -22,7 +22,838 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4986" uniqueCount="4155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5263" uniqueCount="4432">
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>poptot</t>
+  </si>
+  <si>
+    <t>thr</t>
+  </si>
+  <si>
+    <t>topavg</t>
+  </si>
+  <si>
+    <t>bracketavg</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>eff_tax_rate</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
   <si>
     <t>poptot</t>
   </si>
@@ -12539,31 +13370,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4155</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4156</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4157</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4158</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4159</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4160</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4161</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4162</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="2">
@@ -12592,7 +13423,7 @@
         <v>2014</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4164</v>
       </c>
     </row>
     <row r="3">
@@ -12619,7 +13450,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4165</v>
       </c>
     </row>
     <row r="4">
@@ -12646,7 +13477,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4166</v>
       </c>
     </row>
     <row r="5">
@@ -12673,7 +13504,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4167</v>
       </c>
     </row>
     <row r="6">
@@ -12700,7 +13531,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4168</v>
       </c>
     </row>
     <row r="7">
@@ -12727,7 +13558,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4169</v>
       </c>
     </row>
     <row r="8">
@@ -12754,7 +13585,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4170</v>
       </c>
     </row>
     <row r="9">
@@ -12781,7 +13612,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4171</v>
       </c>
     </row>
     <row r="10">
@@ -12808,7 +13639,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4172</v>
       </c>
     </row>
     <row r="11">
@@ -12835,7 +13666,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4173</v>
       </c>
     </row>
     <row r="12">
@@ -12862,7 +13693,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4174</v>
       </c>
     </row>
     <row r="13">
@@ -12889,7 +13720,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4175</v>
       </c>
     </row>
     <row r="14">
@@ -12916,7 +13747,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4176</v>
       </c>
     </row>
     <row r="15">
@@ -12943,7 +13774,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4177</v>
       </c>
     </row>
     <row r="16">
@@ -12970,7 +13801,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4178</v>
       </c>
     </row>
     <row r="17">
@@ -12997,7 +13828,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4179</v>
       </c>
     </row>
     <row r="18">
@@ -13024,7 +13855,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4180</v>
       </c>
     </row>
     <row r="19">
@@ -13051,7 +13882,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4181</v>
       </c>
     </row>
     <row r="20">
@@ -13078,7 +13909,7 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" t="s">
-        <v>4154</v>
+        <v>4182</v>
       </c>
     </row>
     <row r="21">
@@ -13105,7 +13936,7 @@
       </c>
       <c r="H21" s="1"/>
       <c r="I21" t="s">
-        <v>4154</v>
+        <v>4183</v>
       </c>
     </row>
   </sheetData>
@@ -13119,31 +13950,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4404</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4405</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4406</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4407</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4408</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4409</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4410</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4411</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4412</v>
       </c>
     </row>
     <row r="2">
@@ -13172,7 +14003,7 @@
         <v>2023</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4413</v>
       </c>
     </row>
     <row r="3">
@@ -13199,7 +14030,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4414</v>
       </c>
     </row>
     <row r="4">
@@ -13226,7 +14057,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4415</v>
       </c>
     </row>
     <row r="5">
@@ -13253,7 +14084,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4416</v>
       </c>
     </row>
     <row r="6">
@@ -13280,7 +14111,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4417</v>
       </c>
     </row>
     <row r="7">
@@ -13307,7 +14138,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4418</v>
       </c>
     </row>
     <row r="8">
@@ -13334,7 +14165,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4419</v>
       </c>
     </row>
     <row r="9">
@@ -13361,7 +14192,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4420</v>
       </c>
     </row>
     <row r="10">
@@ -13388,7 +14219,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4421</v>
       </c>
     </row>
     <row r="11">
@@ -13415,7 +14246,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4422</v>
       </c>
     </row>
     <row r="12">
@@ -13442,7 +14273,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4423</v>
       </c>
     </row>
     <row r="13">
@@ -13469,7 +14300,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4424</v>
       </c>
     </row>
     <row r="14">
@@ -13496,7 +14327,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4425</v>
       </c>
     </row>
     <row r="15">
@@ -13523,7 +14354,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4426</v>
       </c>
     </row>
     <row r="16">
@@ -13550,7 +14381,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4427</v>
       </c>
     </row>
     <row r="17">
@@ -13577,7 +14408,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4428</v>
       </c>
     </row>
     <row r="18">
@@ -13604,7 +14435,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4429</v>
       </c>
     </row>
     <row r="19">
@@ -13631,7 +14462,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4430</v>
       </c>
     </row>
     <row r="20">
@@ -13658,7 +14489,7 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" t="s">
-        <v>4154</v>
+        <v>4431</v>
       </c>
     </row>
   </sheetData>
@@ -13672,31 +14503,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4184</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4185</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4186</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4187</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4188</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4189</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4190</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4191</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4192</v>
       </c>
     </row>
     <row r="2">
@@ -13725,7 +14556,7 @@
         <v>2015</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4193</v>
       </c>
     </row>
     <row r="3">
@@ -13752,7 +14583,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4194</v>
       </c>
     </row>
     <row r="4">
@@ -13779,7 +14610,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4195</v>
       </c>
     </row>
     <row r="5">
@@ -13806,7 +14637,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4196</v>
       </c>
     </row>
     <row r="6">
@@ -13833,7 +14664,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4197</v>
       </c>
     </row>
     <row r="7">
@@ -13860,7 +14691,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4198</v>
       </c>
     </row>
     <row r="8">
@@ -13887,7 +14718,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4199</v>
       </c>
     </row>
     <row r="9">
@@ -13914,7 +14745,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="10">
@@ -13941,7 +14772,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4201</v>
       </c>
     </row>
     <row r="11">
@@ -13968,7 +14799,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4202</v>
       </c>
     </row>
     <row r="12">
@@ -13995,7 +14826,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4203</v>
       </c>
     </row>
     <row r="13">
@@ -14022,7 +14853,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4204</v>
       </c>
     </row>
     <row r="14">
@@ -14049,7 +14880,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4205</v>
       </c>
     </row>
     <row r="15">
@@ -14076,7 +14907,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4206</v>
       </c>
     </row>
     <row r="16">
@@ -14103,7 +14934,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4207</v>
       </c>
     </row>
     <row r="17">
@@ -14130,7 +14961,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4208</v>
       </c>
     </row>
     <row r="18">
@@ -14157,7 +14988,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4209</v>
       </c>
     </row>
     <row r="19">
@@ -14184,7 +15015,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4210</v>
       </c>
     </row>
     <row r="20">
@@ -14211,7 +15042,7 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" t="s">
-        <v>4154</v>
+        <v>4211</v>
       </c>
     </row>
     <row r="21">
@@ -14238,7 +15069,7 @@
       </c>
       <c r="H21" s="1"/>
       <c r="I21" t="s">
-        <v>4154</v>
+        <v>4212</v>
       </c>
     </row>
   </sheetData>
@@ -14252,31 +15083,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4213</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4214</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4215</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4216</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4217</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4218</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4219</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4220</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4221</v>
       </c>
     </row>
     <row r="2">
@@ -14305,7 +15136,7 @@
         <v>2016</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4222</v>
       </c>
     </row>
     <row r="3">
@@ -14332,7 +15163,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4223</v>
       </c>
     </row>
     <row r="4">
@@ -14359,7 +15190,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4224</v>
       </c>
     </row>
     <row r="5">
@@ -14386,7 +15217,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4225</v>
       </c>
     </row>
     <row r="6">
@@ -14413,7 +15244,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4226</v>
       </c>
     </row>
     <row r="7">
@@ -14440,7 +15271,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4227</v>
       </c>
     </row>
     <row r="8">
@@ -14467,7 +15298,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4228</v>
       </c>
     </row>
     <row r="9">
@@ -14494,7 +15325,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4229</v>
       </c>
     </row>
     <row r="10">
@@ -14521,7 +15352,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4230</v>
       </c>
     </row>
     <row r="11">
@@ -14548,7 +15379,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4231</v>
       </c>
     </row>
     <row r="12">
@@ -14575,7 +15406,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4232</v>
       </c>
     </row>
     <row r="13">
@@ -14602,7 +15433,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4233</v>
       </c>
     </row>
     <row r="14">
@@ -14629,7 +15460,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4234</v>
       </c>
     </row>
     <row r="15">
@@ -14656,7 +15487,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4235</v>
       </c>
     </row>
     <row r="16">
@@ -14683,7 +15514,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4236</v>
       </c>
     </row>
     <row r="17">
@@ -14710,7 +15541,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4237</v>
       </c>
     </row>
     <row r="18">
@@ -14737,7 +15568,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4238</v>
       </c>
     </row>
     <row r="19">
@@ -14764,7 +15595,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4239</v>
       </c>
     </row>
     <row r="20">
@@ -14791,7 +15622,7 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" t="s">
-        <v>4154</v>
+        <v>4240</v>
       </c>
     </row>
     <row r="21">
@@ -14818,7 +15649,7 @@
       </c>
       <c r="H21" s="1"/>
       <c r="I21" t="s">
-        <v>4154</v>
+        <v>4241</v>
       </c>
     </row>
     <row r="22">
@@ -14845,7 +15676,7 @@
       </c>
       <c r="H22" s="1"/>
       <c r="I22" t="s">
-        <v>4154</v>
+        <v>4242</v>
       </c>
     </row>
   </sheetData>
@@ -14859,31 +15690,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4243</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4244</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4245</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4246</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4247</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4248</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4249</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4250</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4251</v>
       </c>
     </row>
     <row r="2">
@@ -14912,7 +15743,7 @@
         <v>2017</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4252</v>
       </c>
     </row>
     <row r="3">
@@ -14939,7 +15770,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4253</v>
       </c>
     </row>
     <row r="4">
@@ -14966,7 +15797,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4254</v>
       </c>
     </row>
     <row r="5">
@@ -14993,7 +15824,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4255</v>
       </c>
     </row>
     <row r="6">
@@ -15020,7 +15851,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4256</v>
       </c>
     </row>
     <row r="7">
@@ -15047,7 +15878,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4257</v>
       </c>
     </row>
     <row r="8">
@@ -15074,7 +15905,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4258</v>
       </c>
     </row>
     <row r="9">
@@ -15101,7 +15932,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4259</v>
       </c>
     </row>
     <row r="10">
@@ -15128,7 +15959,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4260</v>
       </c>
     </row>
     <row r="11">
@@ -15155,7 +15986,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4261</v>
       </c>
     </row>
     <row r="12">
@@ -15182,7 +16013,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4262</v>
       </c>
     </row>
     <row r="13">
@@ -15209,7 +16040,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4263</v>
       </c>
     </row>
     <row r="14">
@@ -15236,7 +16067,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4264</v>
       </c>
     </row>
     <row r="15">
@@ -15263,7 +16094,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4265</v>
       </c>
     </row>
     <row r="16">
@@ -15290,7 +16121,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4266</v>
       </c>
     </row>
     <row r="17">
@@ -15317,7 +16148,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4267</v>
       </c>
     </row>
     <row r="18">
@@ -15344,7 +16175,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4268</v>
       </c>
     </row>
     <row r="19">
@@ -15371,7 +16202,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4269</v>
       </c>
     </row>
     <row r="20">
@@ -15398,7 +16229,7 @@
       </c>
       <c r="H20" s="1"/>
       <c r="I20" t="s">
-        <v>4154</v>
+        <v>4270</v>
       </c>
     </row>
   </sheetData>
@@ -15412,31 +16243,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4271</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4272</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4273</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4274</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4275</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4276</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4277</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4278</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4279</v>
       </c>
     </row>
     <row r="2">
@@ -15465,7 +16296,7 @@
         <v>2018</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4280</v>
       </c>
     </row>
     <row r="3">
@@ -15492,7 +16323,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4281</v>
       </c>
     </row>
     <row r="4">
@@ -15519,7 +16350,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4282</v>
       </c>
     </row>
     <row r="5">
@@ -15546,7 +16377,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4283</v>
       </c>
     </row>
     <row r="6">
@@ -15573,7 +16404,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4284</v>
       </c>
     </row>
     <row r="7">
@@ -15600,7 +16431,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4285</v>
       </c>
     </row>
     <row r="8">
@@ -15627,7 +16458,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4286</v>
       </c>
     </row>
     <row r="9">
@@ -15654,7 +16485,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4287</v>
       </c>
     </row>
     <row r="10">
@@ -15681,7 +16512,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4288</v>
       </c>
     </row>
     <row r="11">
@@ -15708,7 +16539,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4289</v>
       </c>
     </row>
     <row r="12">
@@ -15735,7 +16566,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4290</v>
       </c>
     </row>
     <row r="13">
@@ -15762,7 +16593,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4291</v>
       </c>
     </row>
     <row r="14">
@@ -15789,7 +16620,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4292</v>
       </c>
     </row>
     <row r="15">
@@ -15816,7 +16647,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4293</v>
       </c>
     </row>
     <row r="16">
@@ -15843,7 +16674,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4294</v>
       </c>
     </row>
     <row r="17">
@@ -15870,7 +16701,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4295</v>
       </c>
     </row>
     <row r="18">
@@ -15897,7 +16728,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4296</v>
       </c>
     </row>
     <row r="19">
@@ -15924,7 +16755,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4297</v>
       </c>
     </row>
   </sheetData>
@@ -15938,31 +16769,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4298</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4299</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4300</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4301</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4302</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4303</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4304</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4305</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4306</v>
       </c>
     </row>
     <row r="2">
@@ -15991,7 +16822,7 @@
         <v>2019</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4307</v>
       </c>
     </row>
     <row r="3">
@@ -16018,7 +16849,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4308</v>
       </c>
     </row>
     <row r="4">
@@ -16045,7 +16876,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4309</v>
       </c>
     </row>
     <row r="5">
@@ -16072,7 +16903,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4310</v>
       </c>
     </row>
     <row r="6">
@@ -16099,7 +16930,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4311</v>
       </c>
     </row>
     <row r="7">
@@ -16126,7 +16957,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4312</v>
       </c>
     </row>
     <row r="8">
@@ -16153,7 +16984,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4313</v>
       </c>
     </row>
     <row r="9">
@@ -16180,7 +17011,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4314</v>
       </c>
     </row>
     <row r="10">
@@ -16207,7 +17038,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4315</v>
       </c>
     </row>
     <row r="11">
@@ -16234,7 +17065,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4316</v>
       </c>
     </row>
     <row r="12">
@@ -16261,7 +17092,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4317</v>
       </c>
     </row>
     <row r="13">
@@ -16288,7 +17119,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4318</v>
       </c>
     </row>
     <row r="14">
@@ -16315,7 +17146,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4319</v>
       </c>
     </row>
     <row r="15">
@@ -16342,7 +17173,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4320</v>
       </c>
     </row>
     <row r="16">
@@ -16369,7 +17200,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4321</v>
       </c>
     </row>
     <row r="17">
@@ -16396,7 +17227,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4322</v>
       </c>
     </row>
     <row r="18">
@@ -16423,7 +17254,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4323</v>
       </c>
     </row>
     <row r="19">
@@ -16450,7 +17281,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4324</v>
       </c>
     </row>
   </sheetData>
@@ -16464,31 +17295,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4325</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4326</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4327</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4328</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4329</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4330</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4331</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4332</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4333</v>
       </c>
     </row>
     <row r="2">
@@ -16517,7 +17348,7 @@
         <v>2020</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4334</v>
       </c>
     </row>
     <row r="3">
@@ -16544,7 +17375,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="4">
@@ -16571,7 +17402,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4336</v>
       </c>
     </row>
     <row r="5">
@@ -16598,7 +17429,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4337</v>
       </c>
     </row>
     <row r="6">
@@ -16625,7 +17456,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4338</v>
       </c>
     </row>
     <row r="7">
@@ -16652,7 +17483,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4339</v>
       </c>
     </row>
     <row r="8">
@@ -16679,7 +17510,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4340</v>
       </c>
     </row>
     <row r="9">
@@ -16706,7 +17537,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4341</v>
       </c>
     </row>
     <row r="10">
@@ -16733,7 +17564,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4342</v>
       </c>
     </row>
     <row r="11">
@@ -16760,7 +17591,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4343</v>
       </c>
     </row>
     <row r="12">
@@ -16787,7 +17618,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4344</v>
       </c>
     </row>
     <row r="13">
@@ -16814,7 +17645,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4345</v>
       </c>
     </row>
     <row r="14">
@@ -16841,7 +17672,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4346</v>
       </c>
     </row>
     <row r="15">
@@ -16868,7 +17699,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4347</v>
       </c>
     </row>
     <row r="16">
@@ -16895,7 +17726,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4348</v>
       </c>
     </row>
     <row r="17">
@@ -16922,7 +17753,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4349</v>
       </c>
     </row>
     <row r="18">
@@ -16949,7 +17780,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4350</v>
       </c>
     </row>
   </sheetData>
@@ -16963,31 +17794,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4351</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4352</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4353</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4354</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4355</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4356</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4357</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4358</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4359</v>
       </c>
     </row>
     <row r="2">
@@ -17016,7 +17847,7 @@
         <v>2021</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4360</v>
       </c>
     </row>
     <row r="3">
@@ -17043,7 +17874,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4361</v>
       </c>
     </row>
     <row r="4">
@@ -17070,7 +17901,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4362</v>
       </c>
     </row>
     <row r="5">
@@ -17097,7 +17928,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4363</v>
       </c>
     </row>
     <row r="6">
@@ -17124,7 +17955,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4364</v>
       </c>
     </row>
     <row r="7">
@@ -17151,7 +17982,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4365</v>
       </c>
     </row>
     <row r="8">
@@ -17178,7 +18009,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4366</v>
       </c>
     </row>
     <row r="9">
@@ -17205,7 +18036,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4367</v>
       </c>
     </row>
     <row r="10">
@@ -17232,7 +18063,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4368</v>
       </c>
     </row>
     <row r="11">
@@ -17259,7 +18090,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4369</v>
       </c>
     </row>
     <row r="12">
@@ -17286,7 +18117,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4370</v>
       </c>
     </row>
     <row r="13">
@@ -17313,7 +18144,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4371</v>
       </c>
     </row>
     <row r="14">
@@ -17340,7 +18171,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4372</v>
       </c>
     </row>
     <row r="15">
@@ -17367,7 +18198,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4373</v>
       </c>
     </row>
     <row r="16">
@@ -17394,7 +18225,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4374</v>
       </c>
     </row>
     <row r="17">
@@ -17421,7 +18252,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4375</v>
       </c>
     </row>
     <row r="18">
@@ -17448,7 +18279,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4376</v>
       </c>
     </row>
   </sheetData>
@@ -17462,31 +18293,31 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>4127</v>
+        <v>4377</v>
       </c>
       <c r="B1" t="s">
-        <v>4128</v>
+        <v>4378</v>
       </c>
       <c r="C1" t="s">
-        <v>4129</v>
+        <v>4379</v>
       </c>
       <c r="D1" t="s">
-        <v>4130</v>
+        <v>4380</v>
       </c>
       <c r="E1" t="s">
-        <v>4131</v>
+        <v>4381</v>
       </c>
       <c r="F1" t="s">
-        <v>4132</v>
+        <v>4382</v>
       </c>
       <c r="G1" t="s">
-        <v>4133</v>
+        <v>4383</v>
       </c>
       <c r="H1" t="s">
-        <v>4134</v>
+        <v>4384</v>
       </c>
       <c r="I1" t="s">
-        <v>4135</v>
+        <v>4385</v>
       </c>
     </row>
     <row r="2">
@@ -17515,7 +18346,7 @@
         <v>2022</v>
       </c>
       <c r="I2" t="s">
-        <v>4136</v>
+        <v>4386</v>
       </c>
     </row>
     <row r="3">
@@ -17542,7 +18373,7 @@
       </c>
       <c r="H3" s="1"/>
       <c r="I3" t="s">
-        <v>4154</v>
+        <v>4387</v>
       </c>
     </row>
     <row r="4">
@@ -17569,7 +18400,7 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" t="s">
-        <v>4154</v>
+        <v>4388</v>
       </c>
     </row>
     <row r="5">
@@ -17596,7 +18427,7 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" t="s">
-        <v>4154</v>
+        <v>4389</v>
       </c>
     </row>
     <row r="6">
@@ -17623,7 +18454,7 @@
       </c>
       <c r="H6" s="1"/>
       <c r="I6" t="s">
-        <v>4154</v>
+        <v>4390</v>
       </c>
     </row>
     <row r="7">
@@ -17650,7 +18481,7 @@
       </c>
       <c r="H7" s="1"/>
       <c r="I7" t="s">
-        <v>4154</v>
+        <v>4391</v>
       </c>
     </row>
     <row r="8">
@@ -17677,7 +18508,7 @@
       </c>
       <c r="H8" s="1"/>
       <c r="I8" t="s">
-        <v>4154</v>
+        <v>4392</v>
       </c>
     </row>
     <row r="9">
@@ -17704,7 +18535,7 @@
       </c>
       <c r="H9" s="1"/>
       <c r="I9" t="s">
-        <v>4154</v>
+        <v>4393</v>
       </c>
     </row>
     <row r="10">
@@ -17731,7 +18562,7 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" t="s">
-        <v>4154</v>
+        <v>4394</v>
       </c>
     </row>
     <row r="11">
@@ -17758,7 +18589,7 @@
       </c>
       <c r="H11" s="1"/>
       <c r="I11" t="s">
-        <v>4154</v>
+        <v>4395</v>
       </c>
     </row>
     <row r="12">
@@ -17785,7 +18616,7 @@
       </c>
       <c r="H12" s="1"/>
       <c r="I12" t="s">
-        <v>4154</v>
+        <v>4396</v>
       </c>
     </row>
     <row r="13">
@@ -17812,7 +18643,7 @@
       </c>
       <c r="H13" s="1"/>
       <c r="I13" t="s">
-        <v>4154</v>
+        <v>4397</v>
       </c>
     </row>
     <row r="14">
@@ -17839,7 +18670,7 @@
       </c>
       <c r="H14" s="1"/>
       <c r="I14" t="s">
-        <v>4154</v>
+        <v>4398</v>
       </c>
     </row>
     <row r="15">
@@ -17866,7 +18697,7 @@
       </c>
       <c r="H15" s="1"/>
       <c r="I15" t="s">
-        <v>4154</v>
+        <v>4399</v>
       </c>
     </row>
     <row r="16">
@@ -17893,7 +18724,7 @@
       </c>
       <c r="H16" s="1"/>
       <c r="I16" t="s">
-        <v>4154</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="17">
@@ -17920,7 +18751,7 @@
       </c>
       <c r="H17" s="1"/>
       <c r="I17" t="s">
-        <v>4154</v>
+        <v>4401</v>
       </c>
     </row>
     <row r="18">
@@ -17947,7 +18778,7 @@
       </c>
       <c r="H18" s="1"/>
       <c r="I18" t="s">
-        <v>4154</v>
+        <v>4402</v>
       </c>
     </row>
     <row r="19">
@@ -17974,7 +18805,7 @@
       </c>
       <c r="H19" s="1"/>
       <c r="I19" t="s">
-        <v>4154</v>
+        <v>4403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>